<commit_message>
docs: inventario con columna VALOR (decisión CEO) — valores en repo privado
Opción B del CEO (repo privado, sin cara al público): INVENTARIO-SECRETOS.xlsx
lleva los valores reales. Columna VALOR añadida; JWT_SECRET y MFA_ENC_KEY
precargados. gitleaks allowlist del archivo + regla 12 de CLAUDE.md documenta
la excepción. Se acepta permanencia en historial de git.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/INVENTARIO-SECRETOS.xlsx
+++ b/docs/INVENTARIO-SECRETOS.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEER PRIMERO" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,14 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secretos" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,8 +27,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -40,7 +52,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,7 +61,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,16 +82,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -437,13 +458,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:A40"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>INVENTARIO DE DATOS / API / CLAVES — COMPAS</t>
@@ -454,81 +475,93 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>⚠️ ESTE ARCHIVO NO CONTIENE VALORES DE SECRETOS — a propósito.</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ ESTE ARCHIVO CONTIENE VALORES REALES DE SECRETOS — por decisión del CEO (2026-07-20).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Regla 12 del proyecto: ningún secreto en el repo. gitleaks en CI bloquea. Un secreto en el</t>
+          <t xml:space="preserve">   Contexto: repo PRIVADO, proyecto sin cara al público. Se aceptó conscientemente que:</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   historial de git queda comprometido para siempre (obligaría a rotar todo).</t>
+          <t xml:space="preserve">     - los valores quedan en el HISTORIAL de git (para sacarlos habría que rotarlos), y</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     - gitleaks NO escanea este archivo (allowlist en .gitleaks.toml).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Este archivo es el MAPA: qué secreto existe, para qué, dónde vive (fuente de verdad) y cómo se</t>
+          <t xml:space="preserve">   Por eso: NO hacer público este repo ni compartirlo con terceros sin revisar este archivo.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>obtiene. Los VALORES reales viven SOLO en:</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Render → Environment de cada servicio (fuente de verdad operativa).</t>
+          <t>Hojas: 'Cuentas' (servicios de RODDOS) - 'Secretos' (mapa + columna VALOR para pegar).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Un gestor de contraseñas del CEO (1Password / Bitwarden) para respaldo — RECOMENDADO.</t>
+          <t>La columna 'VALOR (pegar aquí)' es donde acumulas cada valor conforme lo generas (Atlas, AWS...)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • JWT_SECRET y MFA_ENC_KEY: ya generados, en un archivo LOCAL fuera del repo (scratchpad).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • La cadena ADMIN de Atlas: solo en la máquina del CEO; NUNCA en repo ni en logs/chat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Hojas: 'Cuentas' (servicios reutilizados de RODDOS) · 'Secretos' (mapa de claves, sin valores).</t>
-        </is>
-      </c>
-    </row>
+          <t>y desde donde lo copias a Render. JWT_SECRET y MFA_ENC_KEY ya vienen precargados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -541,7 +574,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -551,7 +584,7 @@
     <col width="52" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="28.05" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Servicio</t>
@@ -850,20 +883,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="60" bestFit="1" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="28.05" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Secreto / Clave</t>
@@ -902,6 +936,11 @@
       <c r="H1" s="3" t="inlineStr">
         <is>
           <t>¿Cargado?</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>VALOR (pegar aquí)</t>
         </is>
       </c>
     </row>
@@ -943,7 +982,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Pendiente de cargar en Render</t>
+          <t>Valor en col I; falta pegar en Render</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SEjBWg49duj_rNo56mkR2GHqHjQtfMxxjGXR5Ed0xnIGDVxVz8BaLLfRVGsoyaco</t>
         </is>
       </c>
     </row>
@@ -985,7 +1029,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Pendiente de cargar en Render</t>
+          <t>Valor en col I; falta pegar en Render</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>N-aOOOge4m-FVxigCFtM4OpXjV3U9uWrQJraGiit1Tg=</t>
         </is>
       </c>
     </row>

</xml_diff>